<commit_message>
Lite - Made good excel inputs and outputs
</commit_message>
<xml_diff>
--- a/referencia.xlsx
+++ b/referencia.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>lineal step</t>
   </si>
@@ -69,6 +69,24 @@
   </si>
   <si>
     <t>Estructuras</t>
+  </si>
+  <si>
+    <t>650</t>
+  </si>
+  <si>
+    <t>6500</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>180</t>
   </si>
   <si>
     <t>1,2,3,4,5,6,7</t>
@@ -636,9 +654,25 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="5:20" x14ac:dyDescent="0.25">
-      <c r="E2" s="10"/>
-      <c r="F2" s="11"/>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>23</v>
+      </c>
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
       <c r="I2" s="10"/>
@@ -655,7 +689,7 @@
       <c r="P2" s="10"/>
       <c r="Q2" s="11"/>
       <c r="R2" s="11" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="S2" s="12"/>
       <c r="T2" s="12"/>

</xml_diff>

<commit_message>
Minor fixes in Lite mode
</commit_message>
<xml_diff>
--- a/referencia.xlsx
+++ b/referencia.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
   <si>
     <t>lineal step</t>
   </si>
@@ -71,22 +71,7 @@
     <t>Estructuras</t>
   </si>
   <si>
-    <t>650</t>
-  </si>
-  <si>
-    <t>6500</t>
-  </si>
-  <si>
-    <t>0,5</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>180</t>
+    <t/>
   </si>
   <si>
     <t>1,2,3,4,5,6,7</t>
@@ -659,19 +644,19 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
@@ -680,16 +665,16 @@
       <c r="K2" s="10"/>
       <c r="L2" s="10"/>
       <c r="M2" s="10"/>
-      <c r="N2" s="10">
-        <v>50</v>
-      </c>
-      <c r="O2" s="10">
-        <v>50</v>
+      <c r="N2" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="O2" s="10" t="s">
+        <v>18</v>
       </c>
       <c r="P2" s="10"/>
       <c r="Q2" s="11"/>
       <c r="R2" s="11" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="S2" s="12"/>
       <c r="T2" s="12"/>

</xml_diff>